<commit_message>
Modification du modèle template fiches_stages.xlsx
</commit_message>
<xml_diff>
--- a/fiches_stages.xlsx
+++ b/fiches_stages.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jxk\Downloads\Stage-Manager\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{934B77CF-5187-402A-A79F-067E0773BBE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72216917-1FBF-4460-B743-F8F7A59A17A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Fiches de Stage" sheetId="1" r:id="rId1"/>
+    <sheet name="Fiche de Stages" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -127,9 +127,6 @@
     <t>KOUAKOUSSUI YANN EZECHIEL AYMARD</t>
   </si>
   <si>
-    <t>KOUAME SOURALEH JATHE</t>
-  </si>
-  <si>
     <t>0767150156</t>
   </si>
   <si>
@@ -182,6 +179,9 @@
   </si>
   <si>
     <t>Contact:  0103736385</t>
+  </si>
+  <si>
+    <t>KOUAME SOURALEH JATHE ITHIEL</t>
   </si>
 </sst>
 </file>
@@ -657,22 +657,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2201A784-6425-4129-8B38-8D9FDE9348E6}">
   <dimension ref="A1:K36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="20" customWidth="1"/>
-    <col min="6" max="7" width="8" customWidth="1"/>
-    <col min="8" max="8" width="20" customWidth="1"/>
-    <col min="9" max="9" width="16.33203125" customWidth="1"/>
-    <col min="10" max="11" width="12" customWidth="1"/>
+    <col min="2" max="2" width="26" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" customWidth="1"/>
+    <col min="4" max="4" width="17.88671875" customWidth="1"/>
+    <col min="5" max="5" width="27.44140625" customWidth="1"/>
+    <col min="7" max="7" width="11.5546875" customWidth="1"/>
+    <col min="8" max="8" width="27.21875" customWidth="1"/>
+    <col min="9" max="9" width="23" customWidth="1"/>
+    <col min="10" max="10" width="19.44140625" customWidth="1"/>
+    <col min="11" max="11" width="19.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" ht="18" x14ac:dyDescent="0.35">
       <c r="B1" s="8" t="s">
         <v>0</v>
       </c>
@@ -686,7 +686,7 @@
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
     </row>
-    <row r="2" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B2" s="10" t="s">
         <v>1</v>
       </c>
@@ -697,7 +697,7 @@
       <c r="G2" s="9"/>
       <c r="H2" s="9"/>
       <c r="I2" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J2" s="9"/>
       <c r="K2" s="9"/>
@@ -707,7 +707,7 @@
         <v>2</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="K3" s="3"/>
     </row>
@@ -741,7 +741,7 @@
       </c>
       <c r="G8" s="13"/>
     </row>
-    <row r="9" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>8</v>
       </c>
@@ -776,7 +776,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>1</v>
       </c>
@@ -793,7 +793,7 @@
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>2</v>
       </c>
@@ -810,7 +810,7 @@
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>3</v>
       </c>
@@ -827,7 +827,7 @@
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>4</v>
       </c>
@@ -844,7 +844,7 @@
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>5</v>
       </c>
@@ -861,7 +861,7 @@
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>6</v>
       </c>
@@ -878,7 +878,7 @@
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>7</v>
       </c>
@@ -895,7 +895,7 @@
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>8</v>
       </c>
@@ -912,7 +912,7 @@
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>9</v>
       </c>
@@ -929,7 +929,7 @@
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>10</v>
       </c>
@@ -946,7 +946,7 @@
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>11</v>
       </c>
@@ -963,7 +963,7 @@
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>12</v>
       </c>
@@ -980,7 +980,7 @@
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>13</v>
       </c>
@@ -997,7 +997,7 @@
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>14</v>
       </c>
@@ -1014,7 +1014,7 @@
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>15</v>
       </c>
@@ -1031,7 +1031,7 @@
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
     </row>
-    <row r="25" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>16</v>
       </c>
@@ -1048,43 +1048,43 @@
       <c r="J25" s="1"/>
       <c r="K25" s="1"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>17</v>
       </c>
       <c r="B26" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G26" s="1"/>
       <c r="H26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="I26" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="I26" s="1" t="s">
+      <c r="J26" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="J26" s="1" t="s">
+      <c r="K26" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="K26" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="27" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>18</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
@@ -1096,12 +1096,12 @@
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>19</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
@@ -1113,12 +1113,12 @@
       <c r="J28" s="1"/>
       <c r="K28" s="1"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>20</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
@@ -1130,12 +1130,12 @@
       <c r="J29" s="1"/>
       <c r="K29" s="1"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>21</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
@@ -1147,12 +1147,12 @@
       <c r="J30" s="1"/>
       <c r="K30" s="1"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>22</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
@@ -1164,12 +1164,12 @@
       <c r="J31" s="1"/>
       <c r="K31" s="1"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>23</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
@@ -1181,12 +1181,12 @@
       <c r="J32" s="1"/>
       <c r="K32" s="1"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>24</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
@@ -1198,12 +1198,12 @@
       <c r="J33" s="1"/>
       <c r="K33" s="1"/>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>25</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
@@ -1215,12 +1215,12 @@
       <c r="J34" s="1"/>
       <c r="K34" s="1"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>26</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
@@ -1232,12 +1232,12 @@
       <c r="J35" s="1"/>
       <c r="K35" s="1"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>27</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
@@ -1252,11 +1252,11 @@
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="B1:K1"/>
+    <mergeCell ref="B2:H2"/>
     <mergeCell ref="I2:K2"/>
     <mergeCell ref="I5:K5"/>
-    <mergeCell ref="B2:H2"/>
     <mergeCell ref="F8:G8"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Mise à jour du template
</commit_message>
<xml_diff>
--- a/fiches_stages.xlsx
+++ b/fiches_stages.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jxk\Downloads\Stage-Manager\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72216917-1FBF-4460-B743-F8F7A59A17A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A8FE1F2-E068-4269-9991-CE6E38D03D3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>FICHE DE SITUATION DES STAGES PFE 2025 - 2026</t>
   </si>
@@ -40,9 +40,6 @@
     <t>FILLIERE-CLASSE: SIGL3</t>
   </si>
   <si>
-    <t>Date:</t>
-  </si>
-  <si>
     <t>EN STAGE</t>
   </si>
   <si>
@@ -127,24 +124,6 @@
     <t>KOUAKOUSSUI YANN EZECHIEL AYMARD</t>
   </si>
   <si>
-    <t>0767150156</t>
-  </si>
-  <si>
-    <t>SOCI</t>
-  </si>
-  <si>
-    <t>Cocody</t>
-  </si>
-  <si>
-    <t>0556551820</t>
-  </si>
-  <si>
-    <t>02/04/2026</t>
-  </si>
-  <si>
-    <t>02/07/2026</t>
-  </si>
-  <si>
     <t>LOBA EMMANUELLA VALENCIA</t>
   </si>
   <si>
@@ -182,6 +161,9 @@
   </si>
   <si>
     <t>KOUAME SOURALEH JATHE ITHIEL</t>
+  </si>
+  <si>
+    <t>Date: 02/04/2026</t>
   </si>
 </sst>
 </file>
@@ -697,7 +679,7 @@
       <c r="G2" s="9"/>
       <c r="H2" s="9"/>
       <c r="I2" s="10" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="J2" s="9"/>
       <c r="K2" s="9"/>
@@ -707,7 +689,7 @@
         <v>2</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="K3" s="3"/>
     </row>
@@ -730,58 +712,58 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="C7" s="6"/>
       <c r="I7" s="5"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="F8" s="12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G8" s="13"/>
     </row>
     <row r="9" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="C9" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="D9" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="E9" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="F9" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="G9" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="H9" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="I9" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="J9" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="J9" s="7" t="s">
+      <c r="K9" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="K9" s="7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>1</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -793,12 +775,12 @@
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
     </row>
-    <row r="11" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>2</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
@@ -810,12 +792,12 @@
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
     </row>
-    <row r="12" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>3</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
@@ -827,12 +809,12 @@
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
     </row>
-    <row r="13" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>4</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
@@ -844,12 +826,12 @@
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
     </row>
-    <row r="14" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>5</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
@@ -861,12 +843,12 @@
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
     </row>
-    <row r="15" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>6</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
@@ -878,12 +860,12 @@
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
     </row>
-    <row r="16" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>7</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
@@ -895,12 +877,12 @@
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
     </row>
-    <row r="17" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>8</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
@@ -912,12 +894,12 @@
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
     </row>
-    <row r="18" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>9</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
@@ -929,12 +911,12 @@
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
     </row>
-    <row r="19" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>10</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
@@ -946,12 +928,12 @@
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
     </row>
-    <row r="20" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>11</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
@@ -963,12 +945,12 @@
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
     </row>
-    <row r="21" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>12</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
@@ -980,12 +962,12 @@
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
     </row>
-    <row r="22" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>13</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
@@ -997,12 +979,12 @@
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
     </row>
-    <row r="23" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>14</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
@@ -1014,12 +996,12 @@
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
     </row>
-    <row r="24" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>15</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
@@ -1031,12 +1013,12 @@
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
     </row>
-    <row r="25" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>16</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
@@ -1048,43 +1030,29 @@
       <c r="J25" s="1"/>
       <c r="K25" s="1"/>
     </row>
-    <row r="26" spans="1:11" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>17</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>35</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="C26" s="1"/>
       <c r="D26" s="1"/>
-      <c r="E26" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
       <c r="G26" s="1"/>
-      <c r="H26" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="I26" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="K26" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="K26" s="1"/>
+    </row>
+    <row r="27" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>18</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
@@ -1096,12 +1064,12 @@
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
     </row>
-    <row r="28" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>19</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
@@ -1113,12 +1081,12 @@
       <c r="J28" s="1"/>
       <c r="K28" s="1"/>
     </row>
-    <row r="29" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>20</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
@@ -1130,12 +1098,12 @@
       <c r="J29" s="1"/>
       <c r="K29" s="1"/>
     </row>
-    <row r="30" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>21</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
@@ -1147,12 +1115,12 @@
       <c r="J30" s="1"/>
       <c r="K30" s="1"/>
     </row>
-    <row r="31" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>22</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
@@ -1164,12 +1132,12 @@
       <c r="J31" s="1"/>
       <c r="K31" s="1"/>
     </row>
-    <row r="32" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>23</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
@@ -1181,12 +1149,12 @@
       <c r="J32" s="1"/>
       <c r="K32" s="1"/>
     </row>
-    <row r="33" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>24</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
@@ -1198,12 +1166,12 @@
       <c r="J33" s="1"/>
       <c r="K33" s="1"/>
     </row>
-    <row r="34" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>25</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
@@ -1215,12 +1183,12 @@
       <c r="J34" s="1"/>
       <c r="K34" s="1"/>
     </row>
-    <row r="35" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>26</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
@@ -1232,12 +1200,12 @@
       <c r="J35" s="1"/>
       <c r="K35" s="1"/>
     </row>
-    <row r="36" spans="1:11" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>27</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>

</xml_diff>